<commit_message>
Tue 15 Apr 2025 10:00:01 CST
</commit_message>
<xml_diff>
--- a/计划/2025学习计划.xlsx
+++ b/计划/2025学习计划.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="23840" activeTab="2"/>
+    <workbookView windowHeight="23480" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="28">
   <si>
     <t>早餐</t>
   </si>
@@ -108,6 +108,21 @@
     </r>
   </si>
   <si>
+    <t>胸</t>
+  </si>
+  <si>
+    <t>背</t>
+  </si>
+  <si>
+    <t>腿</t>
+  </si>
+  <si>
+    <t>肩</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <r>
       <rPr>
         <strike/>
@@ -154,51 +169,7 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">1音频/1视频/10技术书/1习题
-</t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>20非技术书</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-1音频/1视频/10技术书/1习题</t>
-    </r>
-  </si>
-  <si>
-    <t>胸</t>
-  </si>
-  <si>
-    <t>背</t>
-  </si>
-  <si>
-    <t>腿</t>
-  </si>
-  <si>
-    <t>肩</t>
+    <t>跑步</t>
   </si>
   <si>
     <t>1音频/1视频/10技术书/1习题
@@ -247,9 +218,6 @@
   </si>
   <si>
     <t>面包</t>
-  </si>
-  <si>
-    <t>跑步</t>
   </si>
   <si>
     <t>三明治</t>
@@ -2400,25 +2368,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -2510,25 +2478,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2608,25 +2576,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2706,25 +2674,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2780,13 +2748,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -3406,25 +3374,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -3516,25 +3484,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3614,25 +3582,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3712,25 +3680,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3786,13 +3754,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -4524,23 +4492,23 @@
       <c r="B13" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="G13" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>8</v>
+      <c r="C13" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -4619,26 +4587,26 @@
       <c r="A20" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>8</v>
+      <c r="B20" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -4717,26 +4685,26 @@
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>9</v>
+      <c r="B27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -4745,20 +4713,25 @@
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="H28" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" customHeight="1" spans="7:7">
+      <c r="G29" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="30" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -4797,18 +4770,21 @@
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
     </row>
-    <row r="34" s="1" customFormat="1" ht="134" customHeight="1" spans="1:4">
+    <row r="34" s="1" customFormat="1" ht="134" customHeight="1" spans="1:5">
       <c r="A34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>9</v>
+      <c r="B34" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -4924,17 +4900,17 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>4</v>
+      <c r="B5" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>13</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>4</v>
@@ -5062,11 +5038,21 @@
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="D14" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="16" s="1" customFormat="1" customHeight="1" spans="1:8">
       <c r="A16" s="2"/>
@@ -5158,7 +5144,9 @@
       <c r="A21" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="2"/>
+      <c r="B21" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -5428,25 +5416,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -5538,25 +5526,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5636,25 +5624,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5734,25 +5722,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5808,13 +5796,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -5914,7 +5902,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5934,25 +5922,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -6009,10 +5997,10 @@
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -6024,11 +6012,11 @@
         <v>1</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -6040,7 +6028,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -6054,25 +6042,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6080,13 +6068,13 @@
         <v>6</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -6158,25 +6146,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6256,7 +6244,7 @@
         <v>3</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>4</v>
@@ -6455,25 +6443,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -6565,25 +6553,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6649,7 +6637,7 @@
         <v>25</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>25</v>
@@ -6683,25 +6671,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6783,25 +6771,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6857,13 +6845,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -7483,25 +7471,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -7593,25 +7581,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7691,25 +7679,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7789,25 +7777,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7863,13 +7851,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">

</xml_diff>

<commit_message>
Wed 31 Dec 2025 15:47:11 CST
</commit_message>
<xml_diff>
--- a/计划/2025学习计划.xlsx
+++ b/计划/2025学习计划.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="23480" activeTab="3"/>
+    <workbookView windowHeight="17240" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,25 @@
     <sheet name="11" sheetId="12" r:id="rId12"/>
     <sheet name="12" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="144525" concurrentCalc="0"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="24">
   <si>
     <t>早餐</t>
   </si>
@@ -56,7 +69,7 @@
         <strike/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -66,7 +79,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -78,7 +91,7 @@
         <strike/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -88,7 +101,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -100,7 +113,7 @@
         <strike/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -123,12 +136,15 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
+    <t>跑步</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <strike/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -138,7 +154,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -150,59 +166,15 @@
         <strike/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>20非技术书</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-1音频/1视频/10技术书/1习题</t>
-    </r>
-  </si>
-  <si>
-    <t>跑步</t>
-  </si>
-  <si>
-    <t>1音频/1视频/10技术书/1习题
-1音频/1视频/10技术书/1习题
-1音频/1视频/10技术书/1习题</t>
-  </si>
-  <si>
-    <t>面条</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="宋体"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
       <t>1音频/1视频/10技术书/1习题</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-20非技术书
-1音频/1视频/10技术书/1习题</t>
-    </r>
+  </si>
+  <si>
+    <t>面条</t>
   </si>
   <si>
     <t>牛肉包子</t>
@@ -220,20 +192,59 @@
     <t>面包</t>
   </si>
   <si>
-    <t>三明治</t>
+    <r>
+      <t>1音频/1视频/10技术书/1习题</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1音频/1视频/10技术书/1习题</t>
+    </r>
   </si>
   <si>
-    <t>火锅</t>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1音频/1视频/10技术书/1习题</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1音频/1视频/10技术书/1习题</t>
+    </r>
   </si>
   <si>
-    <t>素饺子</t>
-  </si>
-  <si>
-    <t>红薯</t>
-  </si>
-  <si>
-    <t>肩
-跑步</t>
+    <t>1音频/1视频/10技术书/1习题
+1音频/1视频/10技术书/1习题</t>
   </si>
 </sst>
 </file>
@@ -250,7 +261,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -258,7 +269,7 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -272,7 +283,7 @@
       <strike/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -280,7 +291,7 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -288,14 +299,14 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -303,7 +314,7 @@
       <b/>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -311,7 +322,7 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -319,7 +330,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -327,7 +338,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -335,14 +346,14 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -350,7 +361,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -358,7 +369,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -366,14 +377,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -381,42 +392,42 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -916,7 +927,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -950,72 +961,69 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1029,6 +1037,13 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
+<customStorage xmlns="https://web.wps.cn/et/2018/main">
+  <book/>
+  <sheets/>
+</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1293,7 +1308,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -1796,7 +1811,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -1865,25 +1880,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -1975,25 +1990,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2073,25 +2088,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2171,25 +2186,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2245,13 +2260,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -2299,7 +2314,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -2368,25 +2383,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -2478,25 +2493,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2576,25 +2591,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2674,25 +2689,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -2748,13 +2763,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -2802,7 +2817,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -2871,25 +2886,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -2981,25 +2996,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3079,25 +3094,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3177,25 +3192,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3251,13 +3266,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -3305,7 +3320,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -3374,25 +3389,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -3484,25 +3499,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3582,25 +3597,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3680,25 +3695,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -3754,13 +3769,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -3808,7 +3823,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -3876,25 +3891,25 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="15" t="s">
+      <c r="B5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -3986,25 +4001,25 @@
       <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H13" s="15" t="s">
+      <c r="B13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4084,25 +4099,25 @@
       <c r="A20" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H20" s="15" t="s">
+      <c r="B20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4182,25 +4197,25 @@
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H27" s="15" t="s">
+      <c r="B27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4256,13 +4271,13 @@
       <c r="A34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="15" t="s">
+      <c r="B34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4311,7 +4326,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -4379,25 +4394,25 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="15" t="s">
+      <c r="B5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4489,25 +4504,25 @@
       <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H13" s="15" t="s">
+      <c r="B13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4587,25 +4602,25 @@
       <c r="A20" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H20" s="15" t="s">
+      <c r="B20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4685,25 +4700,25 @@
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="H27" s="15" t="s">
+      <c r="B27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -4774,13 +4789,13 @@
       <c r="A34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="15" t="s">
+      <c r="B34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>7</v>
       </c>
       <c r="E34" s="1" t="s">
@@ -4832,7 +4847,9 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="5" width="25.5673076923077" style="1" customWidth="1"/>
+    <col min="6" max="6" width="27.5576923076923" style="1" customWidth="1"/>
+    <col min="7" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -4900,26 +4917,26 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>4</v>
+      <c r="B5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -5010,26 +5027,26 @@
       <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>4</v>
+      <c r="B13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5038,20 +5055,20 @@
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="11" t="s">
+      <c r="D14" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="12" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>9</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5118,26 +5135,26 @@
       <c r="A20" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>4</v>
+      <c r="B20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5218,26 +5235,26 @@
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>4</v>
+      <c r="B27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5292,14 +5309,14 @@
       <c r="A34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>4</v>
+      <c r="B34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -5347,7 +5364,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -5415,26 +5432,26 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>15</v>
+      <c r="B5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -5525,26 +5542,26 @@
       <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>15</v>
+      <c r="B13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5623,26 +5640,26 @@
       <c r="A20" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>15</v>
+      <c r="B20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5721,26 +5738,26 @@
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>15</v>
+      <c r="B27" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5795,14 +5812,14 @@
       <c r="A34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>15</v>
+      <c r="B34" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -5851,7 +5868,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -5901,8 +5918,8 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="12" t="s">
-        <v>16</v>
+      <c r="H3" s="13" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -5921,26 +5938,26 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>17</v>
+      <c r="B5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -5996,11 +6013,11 @@
         <v>0</v>
       </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>19</v>
+      <c r="C10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>17</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -6011,12 +6028,12 @@
       <c r="A11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>20</v>
+      <c r="B11" s="12" t="s">
+        <v>18</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="11" t="s">
-        <v>21</v>
+      <c r="D11" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -6027,8 +6044,8 @@
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>22</v>
+      <c r="B12" s="12" t="s">
+        <v>20</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -6041,40 +6058,40 @@
       <c r="A13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>17</v>
+      <c r="B13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
       <c r="A14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="11" t="s">
+      <c r="B14" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="11" t="s">
-        <v>14</v>
+      <c r="D14" s="12" t="s">
+        <v>13</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -6145,26 +6162,26 @@
       <c r="A20" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>17</v>
+      <c r="B20" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>21</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6244,25 +6261,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>4</v>
+        <v>22</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6318,13 +6335,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -6372,7 +6389,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -6409,9 +6426,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="11" t="s">
-        <v>23</v>
-      </c>
+      <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
     <row r="3" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6443,25 +6458,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -6553,25 +6568,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6616,12 +6631,8 @@
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
-      <c r="D17" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>23</v>
-      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -6630,18 +6641,10 @@
       <c r="A18" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>25</v>
-      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -6650,18 +6653,10 @@
       <c r="A19" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>26</v>
-      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -6671,25 +6666,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6698,9 +6693,7 @@
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="13" t="s">
-        <v>27</v>
-      </c>
+      <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -6771,25 +6764,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -6845,13 +6838,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -6899,7 +6892,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -6968,25 +6961,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -7078,25 +7071,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7176,25 +7169,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7274,25 +7267,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7348,13 +7341,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">
@@ -7402,7 +7395,7 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="40" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="18.75" style="1" customWidth="1"/>
-    <col min="2" max="8" width="25.5625" style="1" customWidth="1"/>
+    <col min="2" max="8" width="25.5673076923077" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -7471,25 +7464,25 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="44" customHeight="1" spans="1:8">
@@ -7581,25 +7574,25 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7679,25 +7672,25 @@
         <v>3</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7777,25 +7770,25 @@
         <v>3</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" customHeight="1" spans="1:8">
@@ -7851,13 +7844,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="1" customHeight="1" spans="1:4">

</xml_diff>